<commit_message>
aligned file versions, automatically find newest file version in the app, cleanup, bugfixes
</commit_message>
<xml_diff>
--- a/data/metadata_master_v26.xlsx
+++ b/data/metadata_master_v26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m.arnz\Code\dosi\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EC9CDD-7824-4340-B85D-C863DF85CFE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D399F47-2161-4B56-AB98-3620BBB4A00F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37470" yWindow="-9770" windowWidth="25390" windowHeight="15410" xr2:uid="{B6364C22-E200-354E-9F77-65099374D1D4}"/>
+    <workbookView xWindow="-19300" yWindow="-10700" windowWidth="19390" windowHeight="20970" xr2:uid="{B6364C22-E200-354E-9F77-65099374D1D4}"/>
   </bookViews>
   <sheets>
     <sheet name="metadata labelling" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1453" uniqueCount="1370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1459" uniqueCount="1374">
   <si>
     <t>Innovation Number</t>
   </si>
@@ -4191,6 +4191,18 @@
   </si>
   <si>
     <t>tra</t>
+  </si>
+  <si>
+    <t>LDC</t>
+  </si>
+  <si>
+    <t>LDCs</t>
+  </si>
+  <si>
+    <t>ldc</t>
+  </si>
+  <si>
+    <t>Least Developed Countries</t>
   </si>
 </sst>
 </file>
@@ -6681,7 +6693,7 @@
         <v>129</v>
       </c>
       <c r="H40" s="8" t="str">
-        <f t="shared" ref="H40:H59" si="7">LOWER(LEFT(G40,3))</f>
+        <f t="shared" ref="H40:H61" si="7">LOWER(LEFT(G40,3))</f>
         <v>oce</v>
       </c>
       <c r="I40" t="str">
@@ -7345,6 +7357,19 @@
       </c>
     </row>
     <row r="60" spans="1:23">
+      <c r="G60" s="13" t="s">
+        <v>1370</v>
+      </c>
+      <c r="H60" s="13" t="str">
+        <f t="shared" si="7"/>
+        <v>ldc</v>
+      </c>
+      <c r="I60" s="13" t="s">
+        <v>1372</v>
+      </c>
+      <c r="J60" s="13" t="s">
+        <v>1373</v>
+      </c>
       <c r="R60" t="s">
         <v>737</v>
       </c>
@@ -7359,6 +7384,19 @@
       </c>
     </row>
     <row r="61" spans="1:23">
+      <c r="G61" s="13" t="s">
+        <v>1371</v>
+      </c>
+      <c r="H61" s="13" t="str">
+        <f t="shared" si="7"/>
+        <v>ldc</v>
+      </c>
+      <c r="I61" s="13" t="s">
+        <v>1372</v>
+      </c>
+      <c r="J61" s="13" t="s">
+        <v>1373</v>
+      </c>
       <c r="R61" t="s">
         <v>738</v>
       </c>
@@ -10645,15 +10683,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="c1090911-16f1-4708-addb-5db4084efaec">
@@ -10663,6 +10692,15 @@
     <notes xmlns="c1090911-16f1-4708-addb-5db4084efaec" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -10929,20 +10967,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBA54BCB-AA5D-4698-9843-9222952A1713}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B5CF216-C61E-490A-9803-EEB13155CC39}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="c1090911-16f1-4708-addb-5db4084efaec"/>
     <ds:schemaRef ds:uri="038a7a37-6bdc-40eb-a876-7e5ad11546ed"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DBA54BCB-AA5D-4698-9843-9222952A1713}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>